<commit_message>
Get rid of Our Team page
</commit_message>
<xml_diff>
--- a/news_archive.xlsx
+++ b/news_archive.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10720"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/madisonrichardson/coastwatch-wcn/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80F2DBB4-4100-5548-AA59-C455002FE3F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB1A13BF-4FAD-654F-9286-F2BE46AFCCAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="23220" yWindow="1800" windowWidth="12920" windowHeight="17440" xr2:uid="{4BBD6C59-3026-CA41-B396-04EB3E49D8C4}"/>
   </bookViews>
@@ -49,9 +49,6 @@
     <t>VIIRS POC and PIC Datasets</t>
   </si>
   <si>
-    <t>VIIRS &lt;a href="https://coastwatch.pfeg.noaa.gov/erddap/search/index.html?page=1&amp;itemsPerPage=1000&amp;searchFor=viirs+poc" target="_blank"&gt;POC&lt;/a&gt; and &lt;a href="https://coastwatch.pfeg.noaa.gov/erddap/search/index.html?page=1&amp;itemsPerPage=1000&amp;searchFor=viirs+pic" target="_blank"&gt;PIC&lt;/a&gt; are now available on ERDDAP</t>
-  </si>
-  <si>
     <t>2015 NOAA Ocean Satellite Data Course</t>
   </si>
   <si>
@@ -598,9 +595,6 @@
     <t>Spray Glider Dataset from Scripps</t>
   </si>
   <si>
-    <t>The &lt;a href=“https://coastwatch.pfeg.noaa.gov/wcn/erddap/tabledap/scrippsGlidersSQ.graph” target=“_blank”&gt;Spray Glider dataset&lt;/a&gt; from Scripps Institution of Oceanography is avaialbe for download on ERDDAP.</t>
-  </si>
-  <si>
     <t>New Publication on Alexandrium catenella Blooms</t>
   </si>
   <si>
@@ -617,6 +611,12 @@
   </si>
   <si>
     <t>Job Opportunity: Cloud Specialist</t>
+  </si>
+  <si>
+    <t>VIIRS &lt;a href="https://coastwatch.pfeg.noaa.gov/erddap/search/index.html?page=1&amp;itemsPerPage=1000&amp;searchFor=viirs+poc" target="_blank"&gt;POC&lt;/a&gt; and &lt;a href="https://coastwatch.pfeg.noaa.gov/erddap/search/index.html?page=1&amp;itemsPerPage=1000&amp;searchFor=viirs+pic" target="_blank"&gt;PIC&lt;/a&gt; are now available on ERDDAP.</t>
+  </si>
+  <si>
+    <t>The &lt;a href=“https://coastwatch.pfeg.noaa.gov/wcn/erddap/tabledap/scrippsGlidersSQ.graph” target=“_blank”&gt;Spray Glider dataset&lt;/a&gt; from Scripps Institution of Oceanography is available for download on ERDDAP.</t>
   </si>
 </sst>
 </file>
@@ -999,7 +999,7 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>192</v>
       </c>
       <c r="C2" s="1">
         <v>41877</v>
@@ -1007,10 +1007,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
         <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
       </c>
       <c r="C3" s="1">
         <v>41948</v>
@@ -1018,10 +1018,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
         <v>7</v>
-      </c>
-      <c r="B4" t="s">
-        <v>8</v>
       </c>
       <c r="C4" s="1">
         <v>41948</v>
@@ -1029,10 +1029,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
         <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>10</v>
       </c>
       <c r="C5" s="1">
         <v>42037</v>
@@ -1040,10 +1040,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
         <v>11</v>
-      </c>
-      <c r="B6" t="s">
-        <v>12</v>
       </c>
       <c r="C6" s="1">
         <v>42072</v>
@@ -1051,10 +1051,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
         <v>13</v>
-      </c>
-      <c r="B7" t="s">
-        <v>14</v>
       </c>
       <c r="C7" s="1">
         <v>42297</v>
@@ -1062,10 +1062,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
         <v>15</v>
-      </c>
-      <c r="B8" t="s">
-        <v>16</v>
       </c>
       <c r="C8" s="1">
         <v>42306</v>
@@ -1073,10 +1073,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="s">
         <v>17</v>
-      </c>
-      <c r="B9" t="s">
-        <v>18</v>
       </c>
       <c r="C9" s="1">
         <v>42328</v>
@@ -1084,10 +1084,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" t="s">
         <v>19</v>
-      </c>
-      <c r="B10" t="s">
-        <v>20</v>
       </c>
       <c r="C10" s="1">
         <v>42341</v>
@@ -1095,10 +1095,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" t="s">
         <v>21</v>
-      </c>
-      <c r="B11" t="s">
-        <v>22</v>
       </c>
       <c r="C11" s="1">
         <v>42412</v>
@@ -1106,10 +1106,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" t="s">
         <v>21</v>
-      </c>
-      <c r="B12" t="s">
-        <v>22</v>
       </c>
       <c r="C12" s="1">
         <v>42480</v>
@@ -1117,10 +1117,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" t="s">
         <v>23</v>
-      </c>
-      <c r="B13" t="s">
-        <v>24</v>
       </c>
       <c r="C13" s="1">
         <v>42482</v>
@@ -1128,10 +1128,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C14" s="1">
         <v>42495</v>
@@ -1139,10 +1139,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" t="s">
         <v>26</v>
-      </c>
-      <c r="B15" t="s">
-        <v>27</v>
       </c>
       <c r="C15" s="1">
         <v>42499</v>
@@ -1150,10 +1150,10 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" t="s">
         <v>28</v>
-      </c>
-      <c r="B16" t="s">
-        <v>29</v>
       </c>
       <c r="C16" s="1">
         <v>42499</v>
@@ -1161,10 +1161,10 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B17" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C17" s="1">
         <v>42510</v>
@@ -1172,10 +1172,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" t="s">
         <v>31</v>
-      </c>
-      <c r="B18" t="s">
-        <v>32</v>
       </c>
       <c r="C18" s="1">
         <v>42639</v>
@@ -1183,10 +1183,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19" t="s">
         <v>33</v>
-      </c>
-      <c r="B19" t="s">
-        <v>34</v>
       </c>
       <c r="C19" s="1">
         <v>42646</v>
@@ -1194,10 +1194,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20" t="s">
         <v>35</v>
-      </c>
-      <c r="B20" t="s">
-        <v>36</v>
       </c>
       <c r="C20" s="1">
         <v>42660</v>
@@ -1205,10 +1205,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B21" t="s">
         <v>37</v>
-      </c>
-      <c r="B21" t="s">
-        <v>38</v>
       </c>
       <c r="C21" s="1">
         <v>42709</v>
@@ -1216,10 +1216,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
+        <v>38</v>
+      </c>
+      <c r="B22" t="s">
         <v>39</v>
-      </c>
-      <c r="B22" t="s">
-        <v>40</v>
       </c>
       <c r="C22" s="1">
         <v>42758</v>
@@ -1227,10 +1227,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C23" s="1">
         <v>42849</v>
@@ -1238,10 +1238,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
+        <v>42</v>
+      </c>
+      <c r="B24" t="s">
         <v>43</v>
-      </c>
-      <c r="B24" t="s">
-        <v>44</v>
       </c>
       <c r="C24" s="1">
         <v>42853</v>
@@ -1249,10 +1249,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
+        <v>44</v>
+      </c>
+      <c r="B25" t="s">
         <v>45</v>
-      </c>
-      <c r="B25" t="s">
-        <v>46</v>
       </c>
       <c r="C25" s="1">
         <v>42853</v>
@@ -1260,10 +1260,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26" t="s">
         <v>47</v>
-      </c>
-      <c r="B26" t="s">
-        <v>48</v>
       </c>
       <c r="C26" s="1">
         <v>42895</v>
@@ -1271,10 +1271,10 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B27" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C27" s="1">
         <v>42962</v>
@@ -1282,10 +1282,10 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28" t="s">
         <v>50</v>
-      </c>
-      <c r="B28" t="s">
-        <v>51</v>
       </c>
       <c r="C28" s="1">
         <v>43018</v>
@@ -1293,10 +1293,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
+        <v>51</v>
+      </c>
+      <c r="B29" t="s">
         <v>52</v>
-      </c>
-      <c r="B29" t="s">
-        <v>53</v>
       </c>
       <c r="C29" s="1">
         <v>43019</v>
@@ -1304,10 +1304,10 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
+        <v>53</v>
+      </c>
+      <c r="B30" t="s">
         <v>54</v>
-      </c>
-      <c r="B30" t="s">
-        <v>55</v>
       </c>
       <c r="C30" s="1">
         <v>43027</v>
@@ -1315,10 +1315,10 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
+        <v>55</v>
+      </c>
+      <c r="B31" t="s">
         <v>56</v>
-      </c>
-      <c r="B31" t="s">
-        <v>57</v>
       </c>
       <c r="C31" s="1">
         <v>43046</v>
@@ -1326,10 +1326,10 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
+        <v>57</v>
+      </c>
+      <c r="B32" t="s">
         <v>58</v>
-      </c>
-      <c r="B32" t="s">
-        <v>59</v>
       </c>
       <c r="C32" s="1">
         <v>43046</v>
@@ -1337,10 +1337,10 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
+        <v>59</v>
+      </c>
+      <c r="B33" t="s">
         <v>60</v>
-      </c>
-      <c r="B33" t="s">
-        <v>61</v>
       </c>
       <c r="C33" s="1">
         <v>43059</v>
@@ -1348,10 +1348,10 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
+        <v>61</v>
+      </c>
+      <c r="B34" t="s">
         <v>62</v>
-      </c>
-      <c r="B34" t="s">
-        <v>63</v>
       </c>
       <c r="C34" s="1">
         <v>43102</v>
@@ -1359,10 +1359,10 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B35" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C35" s="1">
         <v>43104</v>
@@ -1370,10 +1370,10 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
+        <v>65</v>
+      </c>
+      <c r="B36" t="s">
         <v>66</v>
-      </c>
-      <c r="B36" t="s">
-        <v>67</v>
       </c>
       <c r="C36" s="1">
         <v>43110</v>
@@ -1381,10 +1381,10 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B37" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C37" s="1">
         <v>43150</v>
@@ -1392,10 +1392,10 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
+        <v>68</v>
+      </c>
+      <c r="B38" t="s">
         <v>69</v>
-      </c>
-      <c r="B38" t="s">
-        <v>70</v>
       </c>
       <c r="C38" s="1">
         <v>43161</v>
@@ -1403,10 +1403,10 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
+        <v>70</v>
+      </c>
+      <c r="B39" t="s">
         <v>71</v>
-      </c>
-      <c r="B39" t="s">
-        <v>72</v>
       </c>
       <c r="C39" s="1">
         <v>43238</v>
@@ -1414,10 +1414,10 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
+        <v>72</v>
+      </c>
+      <c r="B40" t="s">
         <v>73</v>
-      </c>
-      <c r="B40" t="s">
-        <v>74</v>
       </c>
       <c r="C40" s="1">
         <v>43250</v>
@@ -1425,10 +1425,10 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
+        <v>74</v>
+      </c>
+      <c r="B41" t="s">
         <v>75</v>
-      </c>
-      <c r="B41" t="s">
-        <v>76</v>
       </c>
       <c r="C41" s="1">
         <v>43269</v>
@@ -1436,10 +1436,10 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B42" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C42" s="1">
         <v>43348</v>
@@ -1447,10 +1447,10 @@
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
+        <v>77</v>
+      </c>
+      <c r="B43" t="s">
         <v>78</v>
-      </c>
-      <c r="B43" t="s">
-        <v>79</v>
       </c>
       <c r="C43" s="1">
         <v>43398</v>
@@ -1458,10 +1458,10 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
+        <v>79</v>
+      </c>
+      <c r="B44" t="s">
         <v>80</v>
-      </c>
-      <c r="B44" t="s">
-        <v>81</v>
       </c>
       <c r="C44" s="1">
         <v>43493</v>
@@ -1469,10 +1469,10 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B45" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C45" s="1">
         <v>43534</v>
@@ -1480,10 +1480,10 @@
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B46" t="s">
         <v>83</v>
-      </c>
-      <c r="B46" t="s">
-        <v>84</v>
       </c>
       <c r="C46" s="1">
         <v>43575</v>
@@ -1491,10 +1491,10 @@
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B47" t="s">
         <v>85</v>
-      </c>
-      <c r="B47" t="s">
-        <v>86</v>
       </c>
       <c r="C47" s="1">
         <v>43605</v>
@@ -1502,10 +1502,10 @@
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
+        <v>86</v>
+      </c>
+      <c r="B48" t="s">
         <v>87</v>
-      </c>
-      <c r="B48" t="s">
-        <v>88</v>
       </c>
       <c r="C48" s="1">
         <v>43620</v>
@@ -1513,10 +1513,10 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B49" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C49" s="1">
         <v>43644</v>
@@ -1524,10 +1524,10 @@
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B50" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C50" s="1">
         <v>43678</v>
@@ -1535,10 +1535,10 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B51" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C51" s="1">
         <v>43707</v>
@@ -1546,10 +1546,10 @@
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
+        <v>92</v>
+      </c>
+      <c r="B52" t="s">
         <v>93</v>
-      </c>
-      <c r="B52" t="s">
-        <v>94</v>
       </c>
       <c r="C52" s="1">
         <v>43739</v>
@@ -1557,10 +1557,10 @@
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B53" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C53" s="1">
         <v>43753</v>
@@ -1568,10 +1568,10 @@
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
+        <v>96</v>
+      </c>
+      <c r="B54" t="s">
         <v>97</v>
-      </c>
-      <c r="B54" t="s">
-        <v>98</v>
       </c>
       <c r="C54" s="1">
         <v>43760</v>
@@ -1579,10 +1579,10 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B55" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C55" s="1">
         <v>43768</v>
@@ -1590,10 +1590,10 @@
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
+        <v>100</v>
+      </c>
+      <c r="B56" t="s">
         <v>101</v>
-      </c>
-      <c r="B56" t="s">
-        <v>102</v>
       </c>
       <c r="C56" s="1">
         <v>43779</v>
@@ -1601,10 +1601,10 @@
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
+        <v>102</v>
+      </c>
+      <c r="B57" t="s">
         <v>103</v>
-      </c>
-      <c r="B57" t="s">
-        <v>104</v>
       </c>
       <c r="C57" s="1">
         <v>43789</v>
@@ -1612,10 +1612,10 @@
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
+        <v>104</v>
+      </c>
+      <c r="B58" t="s">
         <v>105</v>
-      </c>
-      <c r="B58" t="s">
-        <v>106</v>
       </c>
       <c r="C58" s="1">
         <v>43791</v>
@@ -1623,10 +1623,10 @@
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
+        <v>106</v>
+      </c>
+      <c r="B59" t="s">
         <v>107</v>
-      </c>
-      <c r="B59" t="s">
-        <v>108</v>
       </c>
       <c r="C59" s="1">
         <v>43804</v>
@@ -1634,10 +1634,10 @@
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B60" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C60" s="1">
         <v>43871</v>
@@ -1645,10 +1645,10 @@
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
+        <v>109</v>
+      </c>
+      <c r="B61" t="s">
         <v>110</v>
-      </c>
-      <c r="B61" t="s">
-        <v>111</v>
       </c>
       <c r="C61" s="1">
         <v>43906</v>
@@ -1656,10 +1656,10 @@
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
+        <v>112</v>
+      </c>
+      <c r="B62" t="s">
         <v>113</v>
-      </c>
-      <c r="B62" t="s">
-        <v>114</v>
       </c>
       <c r="C62" s="1">
         <v>43931</v>
@@ -1667,10 +1667,10 @@
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B63" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C63" s="1">
         <v>43975</v>
@@ -1678,10 +1678,10 @@
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
+        <v>116</v>
+      </c>
+      <c r="B64" t="s">
         <v>117</v>
-      </c>
-      <c r="B64" t="s">
-        <v>118</v>
       </c>
       <c r="C64" s="1">
         <v>43977</v>
@@ -1689,10 +1689,10 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
+        <v>118</v>
+      </c>
+      <c r="B65" t="s">
         <v>119</v>
-      </c>
-      <c r="B65" t="s">
-        <v>120</v>
       </c>
       <c r="C65" s="1">
         <v>44063</v>
@@ -1700,10 +1700,10 @@
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
+        <v>120</v>
+      </c>
+      <c r="B66" t="s">
         <v>121</v>
-      </c>
-      <c r="B66" t="s">
-        <v>122</v>
       </c>
       <c r="C66" s="1">
         <v>44063</v>
@@ -1711,10 +1711,10 @@
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
+        <v>122</v>
+      </c>
+      <c r="B67" t="s">
         <v>123</v>
-      </c>
-      <c r="B67" t="s">
-        <v>124</v>
       </c>
       <c r="C67" s="1">
         <v>44123</v>
@@ -1722,10 +1722,10 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
+        <v>124</v>
+      </c>
+      <c r="B68" t="s">
         <v>125</v>
-      </c>
-      <c r="B68" t="s">
-        <v>126</v>
       </c>
       <c r="C68" s="1">
         <v>44175</v>
@@ -1733,10 +1733,10 @@
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B69" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C69" s="1">
         <v>44237</v>
@@ -1744,10 +1744,10 @@
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
+        <v>127</v>
+      </c>
+      <c r="B70" t="s">
         <v>128</v>
-      </c>
-      <c r="B70" t="s">
-        <v>129</v>
       </c>
       <c r="C70" s="1">
         <v>44256</v>
@@ -1755,10 +1755,10 @@
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
+        <v>129</v>
+      </c>
+      <c r="B71" t="s">
         <v>130</v>
-      </c>
-      <c r="B71" t="s">
-        <v>131</v>
       </c>
       <c r="C71" s="1">
         <v>44326</v>
@@ -1766,10 +1766,10 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B72" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C72" s="1">
         <v>44338</v>
@@ -1777,10 +1777,10 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
+        <v>132</v>
+      </c>
+      <c r="B73" t="s">
         <v>133</v>
-      </c>
-      <c r="B73" t="s">
-        <v>134</v>
       </c>
       <c r="C73" s="1">
         <v>44348</v>
@@ -1788,10 +1788,10 @@
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B74" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C74" s="1">
         <v>44350</v>
@@ -1799,10 +1799,10 @@
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B75" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C75" s="1">
         <v>44386</v>
@@ -1810,10 +1810,10 @@
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
+        <v>136</v>
+      </c>
+      <c r="B76" t="s">
         <v>137</v>
-      </c>
-      <c r="B76" t="s">
-        <v>138</v>
       </c>
       <c r="C76" s="1">
         <v>44438</v>
@@ -1821,10 +1821,10 @@
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
+        <v>138</v>
+      </c>
+      <c r="B77" t="s">
         <v>139</v>
-      </c>
-      <c r="B77" t="s">
-        <v>140</v>
       </c>
       <c r="C77" s="1">
         <v>44531</v>
@@ -1832,10 +1832,10 @@
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B78" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C78" s="1">
         <v>44575</v>
@@ -1843,10 +1843,10 @@
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B79" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C79" s="1">
         <v>44579</v>
@@ -1854,10 +1854,10 @@
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B80" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C80" s="1">
         <v>44620</v>
@@ -1865,10 +1865,10 @@
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B81" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C81" s="1">
         <v>44623</v>
@@ -1876,10 +1876,10 @@
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
+        <v>144</v>
+      </c>
+      <c r="B82" t="s">
         <v>145</v>
-      </c>
-      <c r="B82" t="s">
-        <v>146</v>
       </c>
       <c r="C82" s="1">
         <v>44642</v>
@@ -1887,10 +1887,10 @@
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
+        <v>146</v>
+      </c>
+      <c r="B83" t="s">
         <v>147</v>
-      </c>
-      <c r="B83" t="s">
-        <v>148</v>
       </c>
       <c r="C83" s="1">
         <v>44650</v>
@@ -1898,10 +1898,10 @@
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
+        <v>148</v>
+      </c>
+      <c r="B84" t="s">
         <v>149</v>
-      </c>
-      <c r="B84" t="s">
-        <v>150</v>
       </c>
       <c r="C84" s="1">
         <v>44645</v>
@@ -1909,10 +1909,10 @@
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
+        <v>150</v>
+      </c>
+      <c r="B85" t="s">
         <v>151</v>
-      </c>
-      <c r="B85" t="s">
-        <v>152</v>
       </c>
       <c r="C85" s="1">
         <v>44676</v>
@@ -1920,10 +1920,10 @@
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
+        <v>152</v>
+      </c>
+      <c r="B86" t="s">
         <v>153</v>
-      </c>
-      <c r="B86" t="s">
-        <v>154</v>
       </c>
       <c r="C86" s="1">
         <v>44769</v>
@@ -1931,10 +1931,10 @@
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
+        <v>154</v>
+      </c>
+      <c r="B87" t="s">
         <v>155</v>
-      </c>
-      <c r="B87" t="s">
-        <v>156</v>
       </c>
       <c r="C87" s="1">
         <v>44875</v>
@@ -1942,10 +1942,10 @@
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B88" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C88" s="1">
         <v>44910</v>
@@ -1953,10 +1953,10 @@
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
+        <v>157</v>
+      </c>
+      <c r="B89" t="s">
         <v>158</v>
-      </c>
-      <c r="B89" t="s">
-        <v>159</v>
       </c>
       <c r="C89" s="1">
         <v>44970</v>
@@ -1964,10 +1964,10 @@
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
+        <v>159</v>
+      </c>
+      <c r="B90" t="s">
         <v>160</v>
-      </c>
-      <c r="B90" t="s">
-        <v>161</v>
       </c>
       <c r="C90" s="1">
         <v>45071</v>
@@ -1975,10 +1975,10 @@
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
+        <v>161</v>
+      </c>
+      <c r="B91" t="s">
         <v>162</v>
-      </c>
-      <c r="B91" t="s">
-        <v>163</v>
       </c>
       <c r="C91" s="1">
         <v>45160</v>
@@ -1986,10 +1986,10 @@
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
+        <v>163</v>
+      </c>
+      <c r="B92" t="s">
         <v>164</v>
-      </c>
-      <c r="B92" t="s">
-        <v>165</v>
       </c>
       <c r="C92" s="1">
         <v>45170</v>
@@ -1997,10 +1997,10 @@
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
+        <v>165</v>
+      </c>
+      <c r="B93" t="s">
         <v>166</v>
-      </c>
-      <c r="B93" t="s">
-        <v>167</v>
       </c>
       <c r="C93" s="1">
         <v>45413</v>
@@ -2008,10 +2008,10 @@
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
+        <v>167</v>
+      </c>
+      <c r="B94" t="s">
         <v>168</v>
-      </c>
-      <c r="B94" t="s">
-        <v>169</v>
       </c>
       <c r="C94" s="1">
         <v>45436</v>
@@ -2019,10 +2019,10 @@
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
+        <v>169</v>
+      </c>
+      <c r="B95" t="s">
         <v>170</v>
-      </c>
-      <c r="B95" t="s">
-        <v>171</v>
       </c>
       <c r="C95" s="1">
         <v>45448</v>
@@ -2030,10 +2030,10 @@
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
+        <v>171</v>
+      </c>
+      <c r="B96" t="s">
         <v>172</v>
-      </c>
-      <c r="B96" t="s">
-        <v>173</v>
       </c>
       <c r="C96" s="1">
         <v>45474</v>
@@ -2041,10 +2041,10 @@
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B97" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C97" s="1">
         <v>45475</v>
@@ -2052,10 +2052,10 @@
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B98" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C98" s="1">
         <v>45525</v>
@@ -2063,10 +2063,10 @@
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B99" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C99" s="1">
         <v>45587</v>
@@ -2074,10 +2074,10 @@
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B100" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C100" s="1">
         <v>45591</v>
@@ -2085,10 +2085,10 @@
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
+        <v>179</v>
+      </c>
+      <c r="B101" t="s">
         <v>180</v>
-      </c>
-      <c r="B101" t="s">
-        <v>181</v>
       </c>
       <c r="C101" s="1">
         <v>45602</v>
@@ -2096,10 +2096,10 @@
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
+        <v>181</v>
+      </c>
+      <c r="B102" t="s">
         <v>182</v>
-      </c>
-      <c r="B102" t="s">
-        <v>183</v>
       </c>
       <c r="C102" s="1">
         <v>45663</v>
@@ -2107,10 +2107,10 @@
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
+        <v>183</v>
+      </c>
+      <c r="B103" t="s">
         <v>184</v>
-      </c>
-      <c r="B103" t="s">
-        <v>185</v>
       </c>
       <c r="C103" s="1">
         <v>45709</v>
@@ -2118,10 +2118,10 @@
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B104" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="C104" s="1">
         <v>45730</v>
@@ -2129,10 +2129,10 @@
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B105" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C105" s="1">
         <v>45740</v>
@@ -2140,10 +2140,10 @@
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B106" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C106" s="1">
         <v>45835</v>
@@ -2151,10 +2151,10 @@
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
+        <v>188</v>
+      </c>
+      <c r="B107" t="s">
         <v>190</v>
-      </c>
-      <c r="B107" t="s">
-        <v>192</v>
       </c>
       <c r="C107" s="1">
         <v>45835</v>

</xml_diff>